<commit_message>
new docs and features added
</commit_message>
<xml_diff>
--- a/docs/RTM.xlsx
+++ b/docs/RTM.xlsx
@@ -16,160 +16,281 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="49">
-  <si>
-    <t>Req ID</t>
-  </si>
-  <si>
-    <t>Category</t>
-  </si>
-  <si>
-    <t>Requirement Description</t>
-  </si>
-  <si>
-    <t>Decoupled Service</t>
-  </si>
-  <si>
-    <t>Priority</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="49">
   <si>
     <t>Status</t>
   </si>
   <si>
-    <t>REQ-01</t>
-  </si>
-  <si>
-    <t>Identity</t>
-  </si>
-  <si>
-    <t>Support for Vegan/Veg/Egg tiers for named members.</t>
-  </si>
-  <si>
-    <t>Identity-Service</t>
-  </si>
-  <si>
-    <t>P0</t>
-  </si>
-  <si>
-    <t>Sprint 1</t>
-  </si>
-  <si>
-    <t>REQ-02</t>
-  </si>
-  <si>
-    <t>Cuisine</t>
-  </si>
-  <si>
-    <t>Tamil Nadu &amp; Continental as peer-level logic packs.</t>
-  </si>
-  <si>
-    <t>Cuisine-Service</t>
-  </si>
-  <si>
-    <t>REQ-03</t>
-  </si>
-  <si>
-    <t>Ritual</t>
-  </si>
-  <si>
-    <t>Auto-detect Lunar dates (Amavasya/Pournami).</t>
-  </si>
-  <si>
-    <t>Lunar-Service</t>
-  </si>
-  <si>
-    <t>REQ-04</t>
-  </si>
-  <si>
-    <t>Sattvic (No Onion/Garlic) filter on ritual days.</t>
-  </si>
-  <si>
-    <t>REQ-05</t>
-  </si>
-  <si>
-    <t>Inventory</t>
-  </si>
-  <si>
-    <t>Binary "In-Fridge" vs "Market" tracking.</t>
-  </si>
-  <si>
-    <t>Inventory-Service</t>
-  </si>
-  <si>
-    <t>P1</t>
-  </si>
-  <si>
-    <t>Sprint 2</t>
-  </si>
-  <si>
-    <t>REQ-06</t>
-  </si>
-  <si>
-    <t>Output</t>
-  </si>
-  <si>
-    <t>WhatsApp Summary (The "Meal Card") generation.</t>
-  </si>
-  <si>
-    <t>Notify-Service</t>
-  </si>
-  <si>
-    <t>REQ-07</t>
-  </si>
-  <si>
-    <t>Innovation</t>
-  </si>
-  <si>
-    <t>AI "Innovation Lab" for leftover experiments.</t>
-  </si>
-  <si>
-    <t>AI-Lab-Service</t>
-  </si>
-  <si>
-    <t>P2</t>
-  </si>
-  <si>
-    <t>Sprint 3</t>
-  </si>
-  <si>
-    <t>REQ-08</t>
-  </si>
-  <si>
-    <t>Pro</t>
-  </si>
-  <si>
-    <t>Cross-Regional Affinity (Ingredient Momentum).</t>
-  </si>
-  <si>
-    <t>REQ-09</t>
-  </si>
-  <si>
-    <t>Scale</t>
-  </si>
-  <si>
-    <t>Multi-Language selection (English, Tamil, etc.).</t>
-  </si>
-  <si>
-    <t>i18n-Service</t>
-  </si>
-  <si>
-    <t>REQ-10</t>
-  </si>
-  <si>
-    <t>Monetize</t>
-  </si>
-  <si>
-    <t>Enable/Disable features (Free vs Pro).</t>
-  </si>
-  <si>
-    <t>Auth-Gateway</t>
+    <t>BRS ID</t>
+  </si>
+  <si>
+    <t>RS ID</t>
+  </si>
+  <si>
+    <t>FS ID</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>BRS.01</t>
+  </si>
+  <si>
+    <t>RS.101</t>
+  </si>
+  <si>
+    <t>Sc 4</t>
+  </si>
+  <si>
+    <r>
+      <t>Market Intelligence:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Wave 5 / RSI / Momentum price signals.</t>
+    </r>
+  </si>
+  <si>
+    <t>✅ Aligned</t>
+  </si>
+  <si>
+    <t>BRS.02</t>
+  </si>
+  <si>
+    <t>RS.102</t>
+  </si>
+  <si>
+    <t>Sc 2/9</t>
+  </si>
+  <si>
+    <r>
+      <t>Regional Diversity:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Sub-styles (Karaikudi, Punjabi, etc.).</t>
+    </r>
+  </si>
+  <si>
+    <t>BRS.03</t>
+  </si>
+  <si>
+    <t>RS.103</t>
+  </si>
+  <si>
+    <t>Sc 5</t>
+  </si>
+  <si>
+    <r>
+      <t>Zero-Entry UX:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Smart Form purchase confirmation.</t>
+    </r>
+  </si>
+  <si>
+    <t>BRS.04</t>
+  </si>
+  <si>
+    <t>RS.104</t>
+  </si>
+  <si>
+    <t>Sc 6</t>
+  </si>
+  <si>
+    <r>
+      <t>Meal Continuity:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Anchor-to-Remix algorithm.</t>
+    </r>
+  </si>
+  <si>
+    <t>BRS.05</t>
+  </si>
+  <si>
+    <t>RS.105</t>
+  </si>
+  <si>
+    <t>Sc 8</t>
+  </si>
+  <si>
+    <r>
+      <t>Personal Agency:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Choice Carousel (Poha/Oats/Swaps).</t>
+    </r>
+  </si>
+  <si>
+    <t>BRS.06</t>
+  </si>
+  <si>
+    <t>RS.106</t>
+  </si>
+  <si>
+    <r>
+      <t>Cultural Guard:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Fasting/Festival filters (Sattvic).</t>
+    </r>
+  </si>
+  <si>
+    <t>BRS.07</t>
+  </si>
+  <si>
+    <t>RS.107</t>
+  </si>
+  <si>
+    <t>Sc 7</t>
+  </si>
+  <si>
+    <r>
+      <t>Attendance Mgmt:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Headcount and guest tracking.</t>
+    </r>
+  </si>
+  <si>
+    <t>BRS.08</t>
+  </si>
+  <si>
+    <t>RS.108</t>
+  </si>
+  <si>
+    <t>Sc 10</t>
+  </si>
+  <si>
+    <r>
+      <t>Milestones:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Function/Event logic (Birthdays, etc.).</t>
+    </r>
+  </si>
+  <si>
+    <t>BRS.09</t>
+  </si>
+  <si>
+    <t>RS.109</t>
+  </si>
+  <si>
+    <t>Sc A1-A4</t>
+  </si>
+  <si>
+    <r>
+      <t>Admin Control:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> CMS for recipes, logic, and staples.</t>
+    </r>
+  </si>
+  <si>
+    <t>BRS.10</t>
+  </si>
+  <si>
+    <t>RS.110</t>
+  </si>
+  <si>
+    <t>Sc 11</t>
+  </si>
+  <si>
+    <r>
+      <t>Volatility:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Real-time same-day meal pivoting.</t>
+    </r>
+  </si>
+  <si>
+    <t>BRS.11</t>
+  </si>
+  <si>
+    <t>RS.111</t>
+  </si>
+  <si>
+    <t>Vault</t>
+  </si>
+  <si>
+    <r>
+      <t>Transaction Learning:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Store history for smart recommendations.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -180,6 +301,19 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -198,7 +332,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -221,17 +355,41 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -534,7 +692,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
@@ -543,224 +701,219 @@
     <col min="5" max="5" width="18.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="106.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="93.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+      <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="D3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="E3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="B4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="93.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+      <c r="C4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="D4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="E4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="B5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="80.400000000000006" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+      <c r="C5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="80.400000000000006" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+      <c r="E5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="1"/>
+    </row>
+    <row r="7" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="B7" s="3" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="106.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
+      <c r="C7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="E7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="B8" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="C8" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="93.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
+      <c r="D8" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="E8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="B9" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="C9" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="D9" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="E9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="93.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
+      <c r="B10" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C10" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D10" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="93.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
+      <c r="E10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B11" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C11" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D11" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="67.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
+      <c r="E11" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B12" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C12" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D12" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>27</v>
+      <c r="E12" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>